<commit_message>
Add 1684 Ayuman Cup wiki page detailing tournament history, format, and results
</commit_message>
<xml_diff>
--- a/data/List of FLLA World Cup Host Nations(1).xlsx
+++ b/data/List of FLLA World Cup Host Nations(1).xlsx
@@ -113,7 +113,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="38">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -215,6 +215,15 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="49" fontId="5" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="5" fillId="3" borderId="3" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1521,8 +1530,10 @@
           <t>Alzuria</t>
         </is>
       </c>
-      <c r="F25" s="32" t="n">
-        <v>46114</v>
+      <c r="F25" s="35" t="inlineStr">
+        <is>
+          <t>5-3</t>
+        </is>
       </c>
       <c r="G25" s="16" t="inlineStr">
         <is>
@@ -1640,8 +1651,10 @@
           <t>Emara</t>
         </is>
       </c>
-      <c r="F28" s="31" t="n">
-        <v>46114</v>
+      <c r="F28" s="36" t="inlineStr">
+        <is>
+          <t>6-3</t>
+        </is>
       </c>
       <c r="G28" s="27" t="inlineStr">
         <is>
@@ -1678,8 +1691,10 @@
           <t>Lycroa</t>
         </is>
       </c>
-      <c r="F29" s="32" t="n">
-        <v>46054</v>
+      <c r="F29" s="35" t="inlineStr">
+        <is>
+          <t>3-1</t>
+        </is>
       </c>
       <c r="G29" s="16" t="inlineStr">
         <is>
@@ -1780,8 +1795,10 @@
           <t>Estijan</t>
         </is>
       </c>
-      <c r="F32" s="33" t="n">
-        <v>46114</v>
+      <c r="F32" s="37" t="inlineStr">
+        <is>
+          <t>6-3</t>
+        </is>
       </c>
       <c r="G32" s="16" t="inlineStr">
         <is>

</xml_diff>